<commit_message>
visualization remainders and grade values
</commit_message>
<xml_diff>
--- a/factors/dem_factors.xlsx
+++ b/factors/dem_factors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leveophan/diplom_clear/factors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F4570C-EC1C-C34A-A6EA-ACFA233FA1D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C48F6ABF-41C8-CF46-BFBB-9BDF340ED1A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="920" windowWidth="17060" windowHeight="19620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="140" yWindow="920" windowWidth="17060" windowHeight="19720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dem_factors" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,8 @@
     <sheet name="coeff_born_death" sheetId="3" r:id="rId3"/>
     <sheet name="life_expectancy" sheetId="4" r:id="rId4"/>
     <sheet name="woman_child" sheetId="5" r:id="rId5"/>
-    <sheet name="migration_growth" sheetId="6" r:id="rId6"/>
-    <sheet name="man_death_coeffs" sheetId="7" r:id="rId7"/>
+    <sheet name="man_death_coeffs" sheetId="7" r:id="rId6"/>
+    <sheet name="migration_growth" sheetId="6" r:id="rId7"/>
     <sheet name="woman_death_coeffs" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
@@ -27,18 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="47">
   <si>
     <t>Возрастные коэффициенты смертности (на 1000 человек)</t>
   </si>
   <si>
     <t>year</t>
-  </si>
-  <si>
-    <t>0-4</t>
-  </si>
-  <si>
-    <t>5-9</t>
   </si>
   <si>
     <t>10-14</t>
@@ -785,6 +779,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -797,16 +794,13 @@
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1129,40 +1123,40 @@
   <sheetData>
     <row r="1" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="74" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="75" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="74" t="s">
+      <c r="D1" s="75" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="75" t="s">
+      <c r="E1" s="74" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="75" t="s">
+      <c r="F1" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="74" t="s">
+      <c r="G1" s="76" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="75" t="s">
+      <c r="H1" s="76" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="76" t="s">
+      <c r="I1" s="77" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" s="78" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="76" t="s">
+      <c r="L1" s="17" t="s">
         <v>38</v>
-      </c>
-      <c r="I1" s="77" t="s">
-        <v>19</v>
-      </c>
-      <c r="J1" s="78" t="s">
-        <v>17</v>
-      </c>
-      <c r="K1" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1" s="17" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1170,37 +1164,37 @@
         <v>1</v>
       </c>
       <c r="B2" s="79" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="57" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="80" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="57" t="s">
+      <c r="E2" s="79" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="80" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="81" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="82" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="83" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="84" t="s">
+        <v>16</v>
+      </c>
+      <c r="K2" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="80" t="s">
+      <c r="L2" s="17" t="s">
         <v>43</v>
-      </c>
-      <c r="E2" s="79" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="80" t="s">
-        <v>26</v>
-      </c>
-      <c r="G2" s="81" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2" s="82" t="s">
-        <v>23</v>
-      </c>
-      <c r="I2" s="83" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="84" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="L2" s="17" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1234,10 +1228,10 @@
       <c r="J3" s="86">
         <v>1.9</v>
       </c>
-      <c r="K3" s="109">
+      <c r="K3" s="102">
         <v>60</v>
       </c>
-      <c r="L3" s="109">
+      <c r="L3" s="102">
         <v>55</v>
       </c>
     </row>
@@ -1272,10 +1266,10 @@
       <c r="J4" s="87">
         <v>2.2000000000000002</v>
       </c>
-      <c r="K4" s="109">
+      <c r="K4" s="102">
         <v>60</v>
       </c>
-      <c r="L4" s="109">
+      <c r="L4" s="102">
         <v>55</v>
       </c>
     </row>
@@ -1310,10 +1304,10 @@
       <c r="J5" s="88">
         <v>2.1</v>
       </c>
-      <c r="K5" s="109">
+      <c r="K5" s="102">
         <v>60</v>
       </c>
-      <c r="L5" s="109">
+      <c r="L5" s="102">
         <v>55</v>
       </c>
     </row>
@@ -1348,10 +1342,10 @@
       <c r="J6" s="88">
         <v>2.1</v>
       </c>
-      <c r="K6" s="109">
+      <c r="K6" s="102">
         <v>60</v>
       </c>
-      <c r="L6" s="109">
+      <c r="L6" s="102">
         <v>55</v>
       </c>
     </row>
@@ -1386,10 +1380,10 @@
       <c r="J7" s="87">
         <v>1.9</v>
       </c>
-      <c r="K7" s="109">
+      <c r="K7" s="102">
         <v>60</v>
       </c>
-      <c r="L7" s="109">
+      <c r="L7" s="102">
         <v>55</v>
       </c>
     </row>
@@ -1424,10 +1418,10 @@
       <c r="J8" s="86">
         <v>1.7</v>
       </c>
-      <c r="K8" s="109">
+      <c r="K8" s="102">
         <v>60</v>
       </c>
-      <c r="L8" s="109">
+      <c r="L8" s="102">
         <v>55</v>
       </c>
     </row>
@@ -1462,10 +1456,10 @@
       <c r="J9" s="86">
         <v>1.8</v>
       </c>
-      <c r="K9" s="109">
+      <c r="K9" s="102">
         <v>60</v>
       </c>
-      <c r="L9" s="109">
+      <c r="L9" s="102">
         <v>55</v>
       </c>
     </row>
@@ -1500,10 +1494,10 @@
       <c r="J10" s="86">
         <v>1.4</v>
       </c>
-      <c r="K10" s="109">
+      <c r="K10" s="102">
         <v>60</v>
       </c>
-      <c r="L10" s="109">
+      <c r="L10" s="102">
         <v>55</v>
       </c>
     </row>
@@ -1533,15 +1527,15 @@
         <v>77.819999999999993</v>
       </c>
       <c r="I11" s="83" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J11" s="87">
         <v>0.9</v>
       </c>
-      <c r="K11" s="109">
+      <c r="K11" s="102">
         <v>60</v>
       </c>
-      <c r="L11" s="109">
+      <c r="L11" s="102">
         <v>55</v>
       </c>
     </row>
@@ -1576,10 +1570,10 @@
       <c r="J12" s="87">
         <v>1.9</v>
       </c>
-      <c r="K12" s="109" t="s">
-        <v>47</v>
-      </c>
-      <c r="L12" s="109">
+      <c r="K12" s="102" t="s">
+        <v>45</v>
+      </c>
+      <c r="L12" s="102">
         <v>55.5</v>
       </c>
     </row>
@@ -1614,11 +1608,11 @@
       <c r="J13" s="88">
         <v>1.3</v>
       </c>
-      <c r="K13" s="109">
-        <v>61</v>
-      </c>
-      <c r="L13" s="109">
-        <v>56</v>
+      <c r="K13" s="102">
+        <v>60.5</v>
+      </c>
+      <c r="L13" s="102">
+        <v>55.5</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1652,10 +1646,10 @@
       <c r="J14" s="87">
         <v>3.9</v>
       </c>
-      <c r="K14" s="109" t="s">
-        <v>48</v>
-      </c>
-      <c r="L14" s="109">
+      <c r="K14" s="102" t="s">
+        <v>46</v>
+      </c>
+      <c r="L14" s="102">
         <v>56.5</v>
       </c>
     </row>
@@ -1690,11 +1684,11 @@
       <c r="J15" s="87">
         <v>0.4</v>
       </c>
-      <c r="K15" s="109">
-        <v>62</v>
-      </c>
-      <c r="L15" s="109">
-        <v>57</v>
+      <c r="K15" s="102">
+        <v>61.5</v>
+      </c>
+      <c r="L15" s="102">
+        <v>56.5</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1728,11 +1722,11 @@
       <c r="J16" s="87">
         <v>1.4</v>
       </c>
-      <c r="K16" s="109">
-        <v>62.5</v>
-      </c>
-      <c r="L16" s="109">
-        <v>57.5</v>
+      <c r="K16" s="102">
+        <v>63</v>
+      </c>
+      <c r="L16" s="102">
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1766,10 +1760,10 @@
       <c r="J17" s="94">
         <v>1.55531535182507</v>
       </c>
-      <c r="K17" s="109">
+      <c r="K17" s="102">
         <v>63</v>
       </c>
-      <c r="L17" s="109">
+      <c r="L17" s="102">
         <v>58</v>
       </c>
     </row>
@@ -1804,10 +1798,10 @@
       <c r="J18" s="94">
         <v>1.5154657155923399</v>
       </c>
-      <c r="K18" s="109">
+      <c r="K18" s="102">
         <v>63.5</v>
       </c>
-      <c r="L18" s="109">
+      <c r="L18" s="102">
         <v>58.5</v>
       </c>
     </row>
@@ -1842,10 +1836,10 @@
       <c r="J19" s="94">
         <v>1.48526480907527</v>
       </c>
-      <c r="K19" s="109">
+      <c r="K19" s="102">
         <v>64</v>
       </c>
-      <c r="L19" s="109">
+      <c r="L19" s="102">
         <v>59</v>
       </c>
     </row>
@@ -1880,10 +1874,10 @@
       <c r="J20" s="94">
         <v>1.4660729566565001</v>
       </c>
-      <c r="K20" s="109">
+      <c r="K20" s="102">
         <v>64.5</v>
       </c>
-      <c r="L20" s="109">
+      <c r="L20" s="102">
         <v>59.5</v>
       </c>
     </row>
@@ -1918,10 +1912,10 @@
       <c r="J21" s="94">
         <v>1.4717581267473701</v>
       </c>
-      <c r="K21" s="109">
+      <c r="K21" s="102">
         <v>65</v>
       </c>
-      <c r="L21" s="109">
+      <c r="L21" s="102">
         <v>60</v>
       </c>
     </row>
@@ -1956,10 +1950,10 @@
       <c r="J22" s="94">
         <v>1.4779857364634501</v>
       </c>
-      <c r="K22" s="109">
+      <c r="K22" s="102">
         <v>65</v>
       </c>
-      <c r="L22" s="109">
+      <c r="L22" s="102">
         <v>60</v>
       </c>
     </row>
@@ -1994,10 +1988,10 @@
       <c r="J23" s="94">
         <v>1.4847628567758799</v>
       </c>
-      <c r="K23" s="109">
+      <c r="K23" s="102">
         <v>65</v>
       </c>
-      <c r="L23" s="109">
+      <c r="L23" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2032,10 +2026,10 @@
       <c r="J24" s="94">
         <v>1.5026401232921101</v>
       </c>
-      <c r="K24" s="109">
+      <c r="K24" s="102">
         <v>65</v>
       </c>
-      <c r="L24" s="109">
+      <c r="L24" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2070,10 +2064,10 @@
       <c r="J25" s="94">
         <v>1.5092193003093599</v>
       </c>
-      <c r="K25" s="109">
+      <c r="K25" s="102">
         <v>65</v>
       </c>
-      <c r="L25" s="109">
+      <c r="L25" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2108,10 +2102,10 @@
       <c r="J26" s="94">
         <v>1.51560822935829</v>
       </c>
-      <c r="K26" s="109">
+      <c r="K26" s="102">
         <v>65</v>
       </c>
-      <c r="L26" s="109">
+      <c r="L26" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2146,10 +2140,10 @@
       <c r="J27" s="94">
         <v>1.5209576525565001</v>
       </c>
-      <c r="K27" s="109">
+      <c r="K27" s="102">
         <v>65</v>
       </c>
-      <c r="L27" s="109">
+      <c r="L27" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2184,10 +2178,10 @@
       <c r="J28" s="94">
         <v>1.5281785795937599</v>
       </c>
-      <c r="K28" s="109">
+      <c r="K28" s="102">
         <v>65</v>
       </c>
-      <c r="L28" s="109">
+      <c r="L28" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2222,10 +2216,10 @@
       <c r="J29" s="94">
         <v>1.53515461504083</v>
       </c>
-      <c r="K29" s="109">
+      <c r="K29" s="102">
         <v>65</v>
       </c>
-      <c r="L29" s="109">
+      <c r="L29" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2260,10 +2254,10 @@
       <c r="J30" s="94">
         <v>1.5411694120524</v>
       </c>
-      <c r="K30" s="109">
+      <c r="K30" s="102">
         <v>65</v>
       </c>
-      <c r="L30" s="109">
+      <c r="L30" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2298,10 +2292,10 @@
       <c r="J31" s="94">
         <v>1.5475752991884</v>
       </c>
-      <c r="K31" s="109">
+      <c r="K31" s="102">
         <v>65</v>
       </c>
-      <c r="L31" s="109">
+      <c r="L31" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2336,10 +2330,10 @@
       <c r="J32" s="94">
         <v>1.5545054261442299</v>
       </c>
-      <c r="K32" s="109">
+      <c r="K32" s="102">
         <v>65</v>
       </c>
-      <c r="L32" s="109">
+      <c r="L32" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2374,10 +2368,10 @@
       <c r="J33" s="94">
         <v>1.5620399985136999</v>
       </c>
-      <c r="K33" s="109">
+      <c r="K33" s="102">
         <v>65</v>
       </c>
-      <c r="L33" s="109">
+      <c r="L33" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2412,10 +2406,10 @@
       <c r="J34" s="94">
         <v>1.56806107923539</v>
       </c>
-      <c r="K34" s="109">
+      <c r="K34" s="102">
         <v>65</v>
       </c>
-      <c r="L34" s="109">
+      <c r="L34" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2450,10 +2444,10 @@
       <c r="J35" s="94">
         <v>1.57467898982587</v>
       </c>
-      <c r="K35" s="109">
+      <c r="K35" s="102">
         <v>65</v>
       </c>
-      <c r="L35" s="109">
+      <c r="L35" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2488,10 +2482,10 @@
       <c r="J36" s="94">
         <v>1.5819059813846099</v>
       </c>
-      <c r="K36" s="109">
+      <c r="K36" s="102">
         <v>65</v>
       </c>
-      <c r="L36" s="109">
+      <c r="L36" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2526,10 +2520,10 @@
       <c r="J37" s="94">
         <v>1.5898125501757601</v>
       </c>
-      <c r="K37" s="109">
+      <c r="K37" s="102">
         <v>65</v>
       </c>
-      <c r="L37" s="109">
+      <c r="L37" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2564,10 +2558,10 @@
       <c r="J38" s="99">
         <v>1.5962358197333</v>
       </c>
-      <c r="K38" s="109">
+      <c r="K38" s="102">
         <v>65</v>
       </c>
-      <c r="L38" s="109">
+      <c r="L38" s="102">
         <v>60</v>
       </c>
     </row>
@@ -2590,25 +2584,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" s="103"/>
-      <c r="C1" s="103"/>
-      <c r="D1" s="103"/>
+      <c r="A1" s="103" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
     </row>
     <row r="2" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="57" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="57" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="57" t="s">
         <v>28</v>
-      </c>
-      <c r="C2" s="57" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="57" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -3204,21 +3198,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="102" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="103"/>
-      <c r="C1" s="103"/>
+      <c r="A1" s="103" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
     </row>
     <row r="2" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="57" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" s="57" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -3642,21 +3636,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="102" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="104"/>
-      <c r="C1" s="104"/>
+      <c r="A1" s="103" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="105"/>
+      <c r="C1" s="105"/>
     </row>
     <row r="2" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="49" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C2" s="49" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -4076,35 +4070,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="102" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" s="105"/>
+      <c r="A1" s="103" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="106"/>
     </row>
     <row r="2" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="40" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>8</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -4568,6 +4562,724 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
+  <dimension ref="A1:N17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12.5" style="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="12.5" style="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5" style="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="10" width="12.5" style="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5" style="14" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="12.5" style="15" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="107" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="107"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="107"/>
+      <c r="L1" s="108"/>
+      <c r="M1" s="108"/>
+      <c r="N1" s="108"/>
+    </row>
+    <row r="2" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>2010</v>
+      </c>
+      <c r="B3" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="C3" s="4">
+        <v>1.2</v>
+      </c>
+      <c r="D3" s="4">
+        <v>2.5</v>
+      </c>
+      <c r="E3" s="4">
+        <v>4.5</v>
+      </c>
+      <c r="F3" s="4">
+        <v>6.8</v>
+      </c>
+      <c r="G3" s="4">
+        <v>7.9</v>
+      </c>
+      <c r="H3" s="4">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="I3" s="4">
+        <v>13.4</v>
+      </c>
+      <c r="J3" s="4">
+        <v>18.600000000000001</v>
+      </c>
+      <c r="K3" s="4">
+        <v>26.3</v>
+      </c>
+      <c r="L3" s="4">
+        <v>37.1</v>
+      </c>
+      <c r="M3" s="4">
+        <v>49.9</v>
+      </c>
+      <c r="N3" s="4">
+        <v>95.2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>2011</v>
+      </c>
+      <c r="B4" s="6">
+        <v>0.4</v>
+      </c>
+      <c r="C4" s="6">
+        <v>1.2</v>
+      </c>
+      <c r="D4" s="6">
+        <v>2.4</v>
+      </c>
+      <c r="E4" s="6">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="F4" s="6">
+        <v>6.4</v>
+      </c>
+      <c r="G4" s="6">
+        <v>7.7</v>
+      </c>
+      <c r="H4" s="6">
+        <v>9.1</v>
+      </c>
+      <c r="I4" s="6">
+        <v>12.5</v>
+      </c>
+      <c r="J4" s="6">
+        <v>17.100000000000001</v>
+      </c>
+      <c r="K4" s="6">
+        <v>24.7</v>
+      </c>
+      <c r="L4" s="6">
+        <v>35.299999999999997</v>
+      </c>
+      <c r="M4" s="6">
+        <v>45.2</v>
+      </c>
+      <c r="N4" s="7">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>2012</v>
+      </c>
+      <c r="B5" s="6">
+        <v>0.4</v>
+      </c>
+      <c r="C5" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D5" s="6">
+        <v>2.4</v>
+      </c>
+      <c r="E5" s="6">
+        <v>3.8</v>
+      </c>
+      <c r="F5" s="6">
+        <v>6.1</v>
+      </c>
+      <c r="G5" s="6">
+        <v>7.5</v>
+      </c>
+      <c r="H5" s="6">
+        <v>8.6</v>
+      </c>
+      <c r="I5" s="6">
+        <v>11.7</v>
+      </c>
+      <c r="J5" s="6">
+        <v>16.2</v>
+      </c>
+      <c r="K5" s="6">
+        <v>23.3</v>
+      </c>
+      <c r="L5" s="6">
+        <v>33.700000000000003</v>
+      </c>
+      <c r="M5" s="6">
+        <v>42.6</v>
+      </c>
+      <c r="N5" s="6">
+        <v>90.3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>2013</v>
+      </c>
+      <c r="B6" s="6">
+        <v>0.4</v>
+      </c>
+      <c r="C6" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D6" s="6">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E6" s="6">
+        <v>3.6</v>
+      </c>
+      <c r="F6" s="6">
+        <v>5.9</v>
+      </c>
+      <c r="G6" s="6">
+        <v>7.5</v>
+      </c>
+      <c r="H6" s="6">
+        <v>8.5</v>
+      </c>
+      <c r="I6" s="6">
+        <v>11.2</v>
+      </c>
+      <c r="J6" s="6">
+        <v>15.5</v>
+      </c>
+      <c r="K6" s="6">
+        <v>22.1</v>
+      </c>
+      <c r="L6" s="6">
+        <v>32.6</v>
+      </c>
+      <c r="M6" s="6">
+        <v>40.9</v>
+      </c>
+      <c r="N6" s="6">
+        <v>89.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>2014</v>
+      </c>
+      <c r="B7" s="6">
+        <v>0.4</v>
+      </c>
+      <c r="C7" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D7" s="6">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="E7" s="6">
+        <v>3.5</v>
+      </c>
+      <c r="F7" s="6">
+        <v>5.7</v>
+      </c>
+      <c r="G7" s="6">
+        <v>7.8</v>
+      </c>
+      <c r="H7" s="6">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="I7" s="6">
+        <v>11.2</v>
+      </c>
+      <c r="J7" s="6">
+        <v>15.3</v>
+      </c>
+      <c r="K7" s="7">
+        <v>22</v>
+      </c>
+      <c r="L7" s="7">
+        <v>32</v>
+      </c>
+      <c r="M7" s="6">
+        <v>41.4</v>
+      </c>
+      <c r="N7" s="6">
+        <v>90.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>2015</v>
+      </c>
+      <c r="B8" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="C8" s="11">
+        <v>1</v>
+      </c>
+      <c r="D8" s="10">
+        <v>1.9</v>
+      </c>
+      <c r="E8" s="10">
+        <v>3.1</v>
+      </c>
+      <c r="F8" s="10">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="G8" s="10">
+        <v>7.3</v>
+      </c>
+      <c r="H8" s="10">
+        <v>8.6</v>
+      </c>
+      <c r="I8" s="10">
+        <v>10.8</v>
+      </c>
+      <c r="J8" s="11">
+        <v>15</v>
+      </c>
+      <c r="K8" s="10">
+        <v>21.4</v>
+      </c>
+      <c r="L8" s="10">
+        <v>31.6</v>
+      </c>
+      <c r="M8" s="10">
+        <v>41.5</v>
+      </c>
+      <c r="N8" s="10">
+        <v>91.9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>2016</v>
+      </c>
+      <c r="B9" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="C9" s="10">
+        <v>0.9</v>
+      </c>
+      <c r="D9" s="10">
+        <v>1.7</v>
+      </c>
+      <c r="E9" s="10">
+        <v>2.7</v>
+      </c>
+      <c r="F9" s="10">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="G9" s="10">
+        <v>6.9</v>
+      </c>
+      <c r="H9" s="10">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="I9" s="10">
+        <v>10.3</v>
+      </c>
+      <c r="J9" s="10">
+        <v>14.6</v>
+      </c>
+      <c r="K9" s="10">
+        <v>20.7</v>
+      </c>
+      <c r="L9" s="10">
+        <v>31.2</v>
+      </c>
+      <c r="M9" s="10">
+        <v>41.9</v>
+      </c>
+      <c r="N9" s="11">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>2017</v>
+      </c>
+      <c r="B10" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="C10" s="10">
+        <v>0.9</v>
+      </c>
+      <c r="D10" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="E10" s="6">
+        <v>2.4</v>
+      </c>
+      <c r="F10" s="11">
+        <v>4</v>
+      </c>
+      <c r="G10" s="10">
+        <v>6.1</v>
+      </c>
+      <c r="H10" s="10">
+        <v>7.7</v>
+      </c>
+      <c r="I10" s="10">
+        <v>9.4</v>
+      </c>
+      <c r="J10" s="6">
+        <v>13.4</v>
+      </c>
+      <c r="K10" s="10">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="L10" s="10">
+        <v>29.3</v>
+      </c>
+      <c r="M10" s="10">
+        <v>40.1</v>
+      </c>
+      <c r="N10" s="10">
+        <v>87.8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>2018</v>
+      </c>
+      <c r="B11" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="D11" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="E11" s="6">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="F11" s="6">
+        <v>3.7</v>
+      </c>
+      <c r="G11" s="6">
+        <v>5.9</v>
+      </c>
+      <c r="H11" s="6">
+        <v>7.9</v>
+      </c>
+      <c r="I11" s="6">
+        <v>9.6</v>
+      </c>
+      <c r="J11" s="6">
+        <v>13.4</v>
+      </c>
+      <c r="K11" s="6">
+        <v>19.2</v>
+      </c>
+      <c r="L11" s="6">
+        <v>29.3</v>
+      </c>
+      <c r="M11" s="6">
+        <v>40.4</v>
+      </c>
+      <c r="N11" s="6">
+        <v>85.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>2019</v>
+      </c>
+      <c r="B12" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="D12" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="E12" s="7">
+        <v>2</v>
+      </c>
+      <c r="F12" s="6">
+        <v>3.5</v>
+      </c>
+      <c r="G12" s="6">
+        <v>5.6</v>
+      </c>
+      <c r="H12" s="6">
+        <v>7.8</v>
+      </c>
+      <c r="I12" s="6">
+        <v>9.5</v>
+      </c>
+      <c r="J12" s="7">
+        <v>13</v>
+      </c>
+      <c r="K12" s="6">
+        <v>18.7</v>
+      </c>
+      <c r="L12" s="6">
+        <v>28.4</v>
+      </c>
+      <c r="M12" s="6">
+        <v>39.1</v>
+      </c>
+      <c r="N12" s="6">
+        <v>81.8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
+        <v>2020</v>
+      </c>
+      <c r="B13" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="D13" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="E13" s="6">
+        <v>2.1</v>
+      </c>
+      <c r="F13" s="6">
+        <v>3.7</v>
+      </c>
+      <c r="G13" s="6">
+        <v>5.9</v>
+      </c>
+      <c r="H13" s="6">
+        <v>8.5</v>
+      </c>
+      <c r="I13" s="6">
+        <v>10.7</v>
+      </c>
+      <c r="J13" s="6">
+        <v>14.6</v>
+      </c>
+      <c r="K13" s="6">
+        <v>21.2</v>
+      </c>
+      <c r="L13" s="6">
+        <v>32.4</v>
+      </c>
+      <c r="M13" s="6">
+        <v>46.7</v>
+      </c>
+      <c r="N13" s="6">
+        <v>99.8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
+        <v>2021</v>
+      </c>
+      <c r="B14" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="D14" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="E14" s="6">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="F14" s="6">
+        <v>3.8</v>
+      </c>
+      <c r="G14" s="6">
+        <v>6.1</v>
+      </c>
+      <c r="H14" s="6">
+        <v>8.9</v>
+      </c>
+      <c r="I14" s="6">
+        <v>11.6</v>
+      </c>
+      <c r="J14" s="6">
+        <v>15.1</v>
+      </c>
+      <c r="K14" s="6">
+        <v>22.7</v>
+      </c>
+      <c r="L14" s="6">
+        <v>33.6</v>
+      </c>
+      <c r="M14" s="6">
+        <v>49.1</v>
+      </c>
+      <c r="N14" s="6">
+        <v>108.3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
+        <v>2022</v>
+      </c>
+      <c r="B15" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="D15" s="7">
+        <v>2</v>
+      </c>
+      <c r="E15" s="6">
+        <v>2.7</v>
+      </c>
+      <c r="F15" s="6">
+        <v>3.9</v>
+      </c>
+      <c r="G15" s="6">
+        <v>5.8</v>
+      </c>
+      <c r="H15" s="6">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="I15" s="6">
+        <v>10.5</v>
+      </c>
+      <c r="J15" s="6">
+        <v>13.1</v>
+      </c>
+      <c r="K15" s="6">
+        <v>18.8</v>
+      </c>
+      <c r="L15" s="6">
+        <v>27.6</v>
+      </c>
+      <c r="M15" s="6">
+        <v>38.200000000000003</v>
+      </c>
+      <c r="N15" s="6">
+        <v>81.2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
+        <v>2023</v>
+      </c>
+      <c r="B16" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="D16" s="7">
+        <v>2</v>
+      </c>
+      <c r="E16" s="6">
+        <v>3.1</v>
+      </c>
+      <c r="F16" s="6">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="G16" s="6">
+        <v>6.1</v>
+      </c>
+      <c r="H16" s="6">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="I16" s="6">
+        <v>11.2</v>
+      </c>
+      <c r="J16" s="6">
+        <v>13.2</v>
+      </c>
+      <c r="K16" s="7">
+        <v>18</v>
+      </c>
+      <c r="L16" s="6">
+        <v>26.1</v>
+      </c>
+      <c r="M16" s="6">
+        <v>35.9</v>
+      </c>
+      <c r="N16" s="6">
+        <v>69.599999999999994</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -4582,17 +5294,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="102" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="106"/>
+      <c r="A1" s="103" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="109"/>
     </row>
     <row r="2" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -4919,818 +5631,6 @@
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-  </sheetPr>
-  <dimension ref="A1:P17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="12.5" style="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="12.5" style="15" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5" style="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="12" width="12.5" style="15" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.5" style="14" bestFit="1" customWidth="1"/>
-    <col min="14" max="16" width="12.5" style="15" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="107" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
-      <c r="I1" s="108"/>
-      <c r="J1" s="108"/>
-      <c r="K1" s="108"/>
-      <c r="L1" s="108"/>
-      <c r="M1" s="107"/>
-      <c r="N1" s="108"/>
-      <c r="O1" s="108"/>
-      <c r="P1" s="108"/>
-    </row>
-    <row r="2" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="M2" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>2010</v>
-      </c>
-      <c r="B3" s="4">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="C3" s="4">
-        <v>0.4</v>
-      </c>
-      <c r="D3" s="4">
-        <v>0.4</v>
-      </c>
-      <c r="E3" s="4">
-        <v>1.2</v>
-      </c>
-      <c r="F3" s="4">
-        <v>2.5</v>
-      </c>
-      <c r="G3" s="4">
-        <v>4.5</v>
-      </c>
-      <c r="H3" s="4">
-        <v>6.8</v>
-      </c>
-      <c r="I3" s="4">
-        <v>7.9</v>
-      </c>
-      <c r="J3" s="4">
-        <v>9.8000000000000007</v>
-      </c>
-      <c r="K3" s="4">
-        <v>13.4</v>
-      </c>
-      <c r="L3" s="4">
-        <v>18.600000000000001</v>
-      </c>
-      <c r="M3" s="4">
-        <v>26.3</v>
-      </c>
-      <c r="N3" s="4">
-        <v>37.1</v>
-      </c>
-      <c r="O3" s="4">
-        <v>49.9</v>
-      </c>
-      <c r="P3" s="4">
-        <v>95.2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>2011</v>
-      </c>
-      <c r="B4" s="6">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="C4" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="D4" s="6">
-        <v>0.4</v>
-      </c>
-      <c r="E4" s="6">
-        <v>1.2</v>
-      </c>
-      <c r="F4" s="6">
-        <v>2.4</v>
-      </c>
-      <c r="G4" s="6">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="H4" s="6">
-        <v>6.4</v>
-      </c>
-      <c r="I4" s="6">
-        <v>7.7</v>
-      </c>
-      <c r="J4" s="6">
-        <v>9.1</v>
-      </c>
-      <c r="K4" s="6">
-        <v>12.5</v>
-      </c>
-      <c r="L4" s="6">
-        <v>17.100000000000001</v>
-      </c>
-      <c r="M4" s="6">
-        <v>24.7</v>
-      </c>
-      <c r="N4" s="6">
-        <v>35.299999999999997</v>
-      </c>
-      <c r="O4" s="6">
-        <v>45.2</v>
-      </c>
-      <c r="P4" s="7">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>2012</v>
-      </c>
-      <c r="B5" s="6">
-        <v>2.5</v>
-      </c>
-      <c r="C5" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="D5" s="6">
-        <v>0.4</v>
-      </c>
-      <c r="E5" s="6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="F5" s="6">
-        <v>2.4</v>
-      </c>
-      <c r="G5" s="6">
-        <v>3.8</v>
-      </c>
-      <c r="H5" s="6">
-        <v>6.1</v>
-      </c>
-      <c r="I5" s="6">
-        <v>7.5</v>
-      </c>
-      <c r="J5" s="6">
-        <v>8.6</v>
-      </c>
-      <c r="K5" s="6">
-        <v>11.7</v>
-      </c>
-      <c r="L5" s="6">
-        <v>16.2</v>
-      </c>
-      <c r="M5" s="6">
-        <v>23.3</v>
-      </c>
-      <c r="N5" s="6">
-        <v>33.700000000000003</v>
-      </c>
-      <c r="O5" s="6">
-        <v>42.6</v>
-      </c>
-      <c r="P5" s="6">
-        <v>90.3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>2013</v>
-      </c>
-      <c r="B6" s="6">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="C6" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="D6" s="6">
-        <v>0.4</v>
-      </c>
-      <c r="E6" s="6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="F6" s="6">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="G6" s="6">
-        <v>3.6</v>
-      </c>
-      <c r="H6" s="6">
-        <v>5.9</v>
-      </c>
-      <c r="I6" s="6">
-        <v>7.5</v>
-      </c>
-      <c r="J6" s="6">
-        <v>8.5</v>
-      </c>
-      <c r="K6" s="6">
-        <v>11.2</v>
-      </c>
-      <c r="L6" s="6">
-        <v>15.5</v>
-      </c>
-      <c r="M6" s="6">
-        <v>22.1</v>
-      </c>
-      <c r="N6" s="6">
-        <v>32.6</v>
-      </c>
-      <c r="O6" s="6">
-        <v>40.9</v>
-      </c>
-      <c r="P6" s="6">
-        <v>89.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>2014</v>
-      </c>
-      <c r="B7" s="6">
-        <v>2.1</v>
-      </c>
-      <c r="C7" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="D7" s="6">
-        <v>0.4</v>
-      </c>
-      <c r="E7" s="6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="F7" s="6">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="G7" s="6">
-        <v>3.5</v>
-      </c>
-      <c r="H7" s="6">
-        <v>5.7</v>
-      </c>
-      <c r="I7" s="6">
-        <v>7.8</v>
-      </c>
-      <c r="J7" s="6">
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="K7" s="6">
-        <v>11.2</v>
-      </c>
-      <c r="L7" s="6">
-        <v>15.3</v>
-      </c>
-      <c r="M7" s="7">
-        <v>22</v>
-      </c>
-      <c r="N7" s="7">
-        <v>32</v>
-      </c>
-      <c r="O7" s="6">
-        <v>41.4</v>
-      </c>
-      <c r="P7" s="6">
-        <v>90.8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>2015</v>
-      </c>
-      <c r="B8" s="10">
-        <v>1.8</v>
-      </c>
-      <c r="C8" s="10">
-        <v>0.3</v>
-      </c>
-      <c r="D8" s="10">
-        <v>0.3</v>
-      </c>
-      <c r="E8" s="11">
-        <v>1</v>
-      </c>
-      <c r="F8" s="10">
-        <v>1.9</v>
-      </c>
-      <c r="G8" s="10">
-        <v>3.1</v>
-      </c>
-      <c r="H8" s="10">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="I8" s="10">
-        <v>7.3</v>
-      </c>
-      <c r="J8" s="10">
-        <v>8.6</v>
-      </c>
-      <c r="K8" s="10">
-        <v>10.8</v>
-      </c>
-      <c r="L8" s="11">
-        <v>15</v>
-      </c>
-      <c r="M8" s="10">
-        <v>21.4</v>
-      </c>
-      <c r="N8" s="10">
-        <v>31.6</v>
-      </c>
-      <c r="O8" s="10">
-        <v>41.5</v>
-      </c>
-      <c r="P8" s="10">
-        <v>91.9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>2016</v>
-      </c>
-      <c r="B9" s="10">
-        <v>1.6</v>
-      </c>
-      <c r="C9" s="10">
-        <v>0.2</v>
-      </c>
-      <c r="D9" s="10">
-        <v>0.3</v>
-      </c>
-      <c r="E9" s="10">
-        <v>0.9</v>
-      </c>
-      <c r="F9" s="10">
-        <v>1.7</v>
-      </c>
-      <c r="G9" s="10">
-        <v>2.7</v>
-      </c>
-      <c r="H9" s="10">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="I9" s="10">
-        <v>6.9</v>
-      </c>
-      <c r="J9" s="10">
-        <v>8.3000000000000007</v>
-      </c>
-      <c r="K9" s="10">
-        <v>10.3</v>
-      </c>
-      <c r="L9" s="10">
-        <v>14.6</v>
-      </c>
-      <c r="M9" s="10">
-        <v>20.7</v>
-      </c>
-      <c r="N9" s="10">
-        <v>31.2</v>
-      </c>
-      <c r="O9" s="10">
-        <v>41.9</v>
-      </c>
-      <c r="P9" s="11">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>2017</v>
-      </c>
-      <c r="B10" s="10">
-        <v>1.4</v>
-      </c>
-      <c r="C10" s="10">
-        <v>0.2</v>
-      </c>
-      <c r="D10" s="10">
-        <v>0.3</v>
-      </c>
-      <c r="E10" s="10">
-        <v>0.9</v>
-      </c>
-      <c r="F10" s="6">
-        <v>1.5</v>
-      </c>
-      <c r="G10" s="6">
-        <v>2.4</v>
-      </c>
-      <c r="H10" s="11">
-        <v>4</v>
-      </c>
-      <c r="I10" s="10">
-        <v>6.1</v>
-      </c>
-      <c r="J10" s="10">
-        <v>7.7</v>
-      </c>
-      <c r="K10" s="10">
-        <v>9.4</v>
-      </c>
-      <c r="L10" s="6">
-        <v>13.4</v>
-      </c>
-      <c r="M10" s="10">
-        <v>19.399999999999999</v>
-      </c>
-      <c r="N10" s="10">
-        <v>29.3</v>
-      </c>
-      <c r="O10" s="10">
-        <v>40.1</v>
-      </c>
-      <c r="P10" s="10">
-        <v>87.8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>2018</v>
-      </c>
-      <c r="B11" s="6">
-        <v>1.3</v>
-      </c>
-      <c r="C11" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="D11" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="E11" s="6">
-        <v>0.8</v>
-      </c>
-      <c r="F11" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="G11" s="6">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="H11" s="6">
-        <v>3.7</v>
-      </c>
-      <c r="I11" s="6">
-        <v>5.9</v>
-      </c>
-      <c r="J11" s="6">
-        <v>7.9</v>
-      </c>
-      <c r="K11" s="6">
-        <v>9.6</v>
-      </c>
-      <c r="L11" s="6">
-        <v>13.4</v>
-      </c>
-      <c r="M11" s="6">
-        <v>19.2</v>
-      </c>
-      <c r="N11" s="6">
-        <v>29.3</v>
-      </c>
-      <c r="O11" s="6">
-        <v>40.4</v>
-      </c>
-      <c r="P11" s="6">
-        <v>85.4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>2019</v>
-      </c>
-      <c r="B12" s="6">
-        <v>1.2</v>
-      </c>
-      <c r="C12" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="D12" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="E12" s="6">
-        <v>0.8</v>
-      </c>
-      <c r="F12" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="G12" s="7">
-        <v>2</v>
-      </c>
-      <c r="H12" s="6">
-        <v>3.5</v>
-      </c>
-      <c r="I12" s="6">
-        <v>5.6</v>
-      </c>
-      <c r="J12" s="6">
-        <v>7.8</v>
-      </c>
-      <c r="K12" s="6">
-        <v>9.5</v>
-      </c>
-      <c r="L12" s="7">
-        <v>13</v>
-      </c>
-      <c r="M12" s="6">
-        <v>18.7</v>
-      </c>
-      <c r="N12" s="6">
-        <v>28.4</v>
-      </c>
-      <c r="O12" s="6">
-        <v>39.1</v>
-      </c>
-      <c r="P12" s="6">
-        <v>81.8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>2020</v>
-      </c>
-      <c r="B13" s="6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="C13" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="D13" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="E13" s="6">
-        <v>0.8</v>
-      </c>
-      <c r="F13" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="G13" s="6">
-        <v>2.1</v>
-      </c>
-      <c r="H13" s="6">
-        <v>3.7</v>
-      </c>
-      <c r="I13" s="6">
-        <v>5.9</v>
-      </c>
-      <c r="J13" s="6">
-        <v>8.5</v>
-      </c>
-      <c r="K13" s="6">
-        <v>10.7</v>
-      </c>
-      <c r="L13" s="6">
-        <v>14.6</v>
-      </c>
-      <c r="M13" s="6">
-        <v>21.2</v>
-      </c>
-      <c r="N13" s="6">
-        <v>32.4</v>
-      </c>
-      <c r="O13" s="6">
-        <v>46.7</v>
-      </c>
-      <c r="P13" s="6">
-        <v>99.8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>2021</v>
-      </c>
-      <c r="B14" s="6">
-        <v>1.2</v>
-      </c>
-      <c r="C14" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="D14" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="E14" s="6">
-        <v>0.8</v>
-      </c>
-      <c r="F14" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="G14" s="6">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="H14" s="6">
-        <v>3.8</v>
-      </c>
-      <c r="I14" s="6">
-        <v>6.1</v>
-      </c>
-      <c r="J14" s="6">
-        <v>8.9</v>
-      </c>
-      <c r="K14" s="6">
-        <v>11.6</v>
-      </c>
-      <c r="L14" s="6">
-        <v>15.1</v>
-      </c>
-      <c r="M14" s="6">
-        <v>22.7</v>
-      </c>
-      <c r="N14" s="6">
-        <v>33.6</v>
-      </c>
-      <c r="O14" s="6">
-        <v>49.1</v>
-      </c>
-      <c r="P14" s="6">
-        <v>108.3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>2022</v>
-      </c>
-      <c r="B15" s="6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="C15" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="D15" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="E15" s="6">
-        <v>0.8</v>
-      </c>
-      <c r="F15" s="7">
-        <v>2</v>
-      </c>
-      <c r="G15" s="6">
-        <v>2.7</v>
-      </c>
-      <c r="H15" s="6">
-        <v>3.9</v>
-      </c>
-      <c r="I15" s="6">
-        <v>5.8</v>
-      </c>
-      <c r="J15" s="6">
-        <v>8.1999999999999993</v>
-      </c>
-      <c r="K15" s="6">
-        <v>10.5</v>
-      </c>
-      <c r="L15" s="6">
-        <v>13.1</v>
-      </c>
-      <c r="M15" s="6">
-        <v>18.8</v>
-      </c>
-      <c r="N15" s="6">
-        <v>27.6</v>
-      </c>
-      <c r="O15" s="6">
-        <v>38.200000000000003</v>
-      </c>
-      <c r="P15" s="6">
-        <v>81.2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>2023</v>
-      </c>
-      <c r="B16" s="6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="C16" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="D16" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="E16" s="6">
-        <v>0.7</v>
-      </c>
-      <c r="F16" s="7">
-        <v>2</v>
-      </c>
-      <c r="G16" s="6">
-        <v>3.1</v>
-      </c>
-      <c r="H16" s="6">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="I16" s="6">
-        <v>6.1</v>
-      </c>
-      <c r="J16" s="6">
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="K16" s="6">
-        <v>11.2</v>
-      </c>
-      <c r="L16" s="6">
-        <v>13.2</v>
-      </c>
-      <c r="M16" s="7">
-        <v>18</v>
-      </c>
-      <c r="N16" s="6">
-        <v>26.1</v>
-      </c>
-      <c r="O16" s="6">
-        <v>35.9</v>
-      </c>
-      <c r="P16" s="6">
-        <v>69.599999999999994</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:P1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5741,14 +5641,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" style="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="16" width="12.5" style="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="14" width="12.5" style="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="107" t="s">
         <v>0</v>
       </c>
@@ -5765,10 +5665,8 @@
       <c r="L1" s="108"/>
       <c r="M1" s="108"/>
       <c r="N1" s="108"/>
-      <c r="O1" s="108"/>
-      <c r="P1" s="108"/>
-    </row>
-    <row r="2" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -5811,714 +5709,624 @@
       <c r="N2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2010</v>
       </c>
       <c r="B3" s="4">
+        <v>0.3</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0.8</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1.3</v>
+      </c>
+      <c r="F3" s="4">
         <v>1.9</v>
       </c>
-      <c r="C3" s="4">
-        <v>0.2</v>
-      </c>
-      <c r="D3" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="E3" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="F3" s="4">
-        <v>0.8</v>
-      </c>
       <c r="G3" s="4">
-        <v>1.3</v>
+        <v>2.4</v>
       </c>
       <c r="H3" s="4">
-        <v>1.9</v>
+        <v>3.2</v>
       </c>
       <c r="I3" s="4">
-        <v>2.4</v>
+        <v>4.2</v>
       </c>
       <c r="J3" s="4">
-        <v>3.2</v>
+        <v>5.9</v>
       </c>
       <c r="K3" s="4">
-        <v>4.2</v>
+        <v>9.1</v>
       </c>
       <c r="L3" s="4">
-        <v>5.9</v>
+        <v>13.1</v>
       </c>
       <c r="M3" s="4">
-        <v>9.1</v>
-      </c>
-      <c r="N3" s="4">
-        <v>13.1</v>
-      </c>
-      <c r="O3" s="4">
         <v>20.100000000000001</v>
       </c>
-      <c r="P3" s="5">
+      <c r="N3" s="5">
         <v>69.8</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>2011</v>
       </c>
       <c r="B4" s="6">
-        <v>1.7</v>
+        <v>0.2</v>
       </c>
       <c r="C4" s="6">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="D4" s="6">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="E4" s="6">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="F4" s="6">
-        <v>0.7</v>
+        <v>1.9</v>
       </c>
       <c r="G4" s="6">
-        <v>1.2</v>
-      </c>
-      <c r="H4" s="6">
-        <v>1.9</v>
-      </c>
-      <c r="I4" s="6">
         <v>2.4</v>
       </c>
-      <c r="J4" s="7">
+      <c r="H4" s="7">
         <v>3</v>
       </c>
-      <c r="K4" s="7">
+      <c r="I4" s="7">
         <v>4</v>
       </c>
+      <c r="J4" s="6">
+        <v>5.6</v>
+      </c>
+      <c r="K4" s="6">
+        <v>8.4</v>
+      </c>
       <c r="L4" s="6">
-        <v>5.6</v>
+        <v>12.4</v>
       </c>
       <c r="M4" s="6">
-        <v>8.4</v>
-      </c>
-      <c r="N4" s="6">
-        <v>12.4</v>
-      </c>
-      <c r="O4" s="6">
         <v>18.5</v>
       </c>
-      <c r="P4" s="8">
+      <c r="N4" s="8">
         <v>65.5</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>2012</v>
       </c>
       <c r="B5" s="6">
-        <v>2.1</v>
+        <v>0.2</v>
       </c>
       <c r="C5" s="6">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="D5" s="6">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="E5" s="6">
-        <v>0.5</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="F5" s="6">
-        <v>0.7</v>
+        <v>1.8</v>
       </c>
       <c r="G5" s="6">
-        <v>1.1000000000000001</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="H5" s="6">
-        <v>1.8</v>
+        <v>2.9</v>
       </c>
       <c r="I5" s="6">
-        <v>2.2999999999999998</v>
+        <v>3.8</v>
       </c>
       <c r="J5" s="6">
-        <v>2.9</v>
-      </c>
-      <c r="K5" s="6">
-        <v>3.8</v>
+        <v>5.3</v>
+      </c>
+      <c r="K5" s="7">
+        <v>8</v>
       </c>
       <c r="L5" s="6">
-        <v>5.3</v>
-      </c>
-      <c r="M5" s="7">
-        <v>8</v>
-      </c>
-      <c r="N5" s="6">
         <v>11.8</v>
       </c>
-      <c r="O5" s="6">
+      <c r="M5" s="6">
         <v>17.2</v>
       </c>
-      <c r="P5" s="8">
+      <c r="N5" s="8">
         <v>66.400000000000006</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>2013</v>
       </c>
       <c r="B6" s="6">
-        <v>1.9</v>
+        <v>0.2</v>
       </c>
       <c r="C6" s="6">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="D6" s="6">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="E6" s="6">
-        <v>0.4</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="F6" s="6">
-        <v>0.6</v>
+        <v>1.8</v>
       </c>
       <c r="G6" s="6">
-        <v>1.1000000000000001</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="H6" s="6">
-        <v>1.8</v>
+        <v>2.9</v>
       </c>
       <c r="I6" s="6">
-        <v>2.2999999999999998</v>
+        <v>3.7</v>
       </c>
       <c r="J6" s="6">
-        <v>2.9</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="K6" s="6">
-        <v>3.7</v>
+        <v>7.7</v>
       </c>
       <c r="L6" s="6">
-        <v>5.0999999999999996</v>
+        <v>11.4</v>
       </c>
       <c r="M6" s="6">
-        <v>7.7</v>
-      </c>
-      <c r="N6" s="6">
-        <v>11.4</v>
-      </c>
-      <c r="O6" s="6">
         <v>16.600000000000001</v>
       </c>
-      <c r="P6" s="9">
+      <c r="N6" s="9">
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>2014</v>
       </c>
       <c r="B7" s="6">
-        <v>1.7</v>
+        <v>0.2</v>
       </c>
       <c r="C7" s="6">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="D7" s="6">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="E7" s="6">
-        <v>0.5</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="F7" s="6">
-        <v>0.6</v>
+        <v>1.8</v>
       </c>
       <c r="G7" s="6">
-        <v>1.1000000000000001</v>
+        <v>2.4</v>
       </c>
       <c r="H7" s="6">
-        <v>1.8</v>
+        <v>2.9</v>
       </c>
       <c r="I7" s="6">
-        <v>2.4</v>
+        <v>3.8</v>
       </c>
       <c r="J7" s="6">
-        <v>2.9</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="K7" s="6">
-        <v>3.8</v>
+        <v>7.6</v>
       </c>
       <c r="L7" s="6">
-        <v>5.0999999999999996</v>
+        <v>11.2</v>
       </c>
       <c r="M7" s="6">
-        <v>7.6</v>
-      </c>
-      <c r="N7" s="6">
-        <v>11.2</v>
-      </c>
-      <c r="O7" s="6">
         <v>16.600000000000001</v>
       </c>
-      <c r="P7" s="8">
+      <c r="N7" s="8">
         <v>68.599999999999994</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>2015</v>
       </c>
       <c r="B8" s="10">
-        <v>1.5</v>
+        <v>0.2</v>
       </c>
       <c r="C8" s="10">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="D8" s="10">
-        <v>0.2</v>
-      </c>
-      <c r="E8" s="10">
-        <v>0.4</v>
+        <v>0.6</v>
+      </c>
+      <c r="E8" s="11">
+        <v>1</v>
       </c>
       <c r="F8" s="10">
-        <v>0.6</v>
-      </c>
-      <c r="G8" s="11">
-        <v>1</v>
+        <v>1.7</v>
+      </c>
+      <c r="G8" s="10">
+        <v>2.4</v>
       </c>
       <c r="H8" s="10">
-        <v>1.7</v>
+        <v>2.9</v>
       </c>
       <c r="I8" s="10">
-        <v>2.4</v>
-      </c>
-      <c r="J8" s="10">
-        <v>2.9</v>
+        <v>3.7</v>
+      </c>
+      <c r="J8" s="11">
+        <v>5</v>
       </c>
       <c r="K8" s="10">
-        <v>3.7</v>
+        <v>7.4</v>
       </c>
       <c r="L8" s="11">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="M8" s="10">
-        <v>7.4</v>
-      </c>
-      <c r="N8" s="11">
-        <v>11</v>
-      </c>
-      <c r="O8" s="10">
         <v>16.600000000000001</v>
       </c>
-      <c r="P8" s="12">
+      <c r="N8" s="12">
         <v>70.8</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>2016</v>
       </c>
       <c r="B9" s="10">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
       <c r="C9" s="10">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="D9" s="10">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="E9" s="10">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="F9" s="10">
-        <v>0.5</v>
+        <v>1.6</v>
       </c>
       <c r="G9" s="10">
-        <v>0.9</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="H9" s="10">
-        <v>1.6</v>
+        <v>2.8</v>
       </c>
       <c r="I9" s="10">
-        <v>2.2999999999999998</v>
+        <v>3.6</v>
       </c>
       <c r="J9" s="10">
-        <v>2.8</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="K9" s="10">
-        <v>3.6</v>
+        <v>7.2</v>
       </c>
       <c r="L9" s="10">
-        <v>4.9000000000000004</v>
+        <v>10.7</v>
       </c>
       <c r="M9" s="10">
-        <v>7.2</v>
-      </c>
-      <c r="N9" s="10">
-        <v>10.7</v>
-      </c>
-      <c r="O9" s="10">
         <v>16.7</v>
       </c>
-      <c r="P9" s="12">
+      <c r="N9" s="12">
         <v>70.8</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>2017</v>
       </c>
-      <c r="B10" s="6">
-        <v>1.1000000000000001</v>
+      <c r="B10" s="10">
+        <v>0.2</v>
       </c>
       <c r="C10" s="10">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="D10" s="10">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="E10" s="10">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="F10" s="10">
-        <v>0.5</v>
+        <v>1.4</v>
       </c>
       <c r="G10" s="10">
-        <v>0.8</v>
+        <v>2.1</v>
       </c>
       <c r="H10" s="10">
-        <v>1.4</v>
+        <v>2.7</v>
       </c>
       <c r="I10" s="10">
-        <v>2.1</v>
+        <v>3.4</v>
       </c>
       <c r="J10" s="10">
-        <v>2.7</v>
+        <v>4.5</v>
       </c>
       <c r="K10" s="10">
-        <v>3.4</v>
+        <v>6.8</v>
       </c>
       <c r="L10" s="10">
-        <v>4.5</v>
+        <v>10.1</v>
       </c>
       <c r="M10" s="10">
-        <v>6.8</v>
-      </c>
-      <c r="N10" s="10">
-        <v>10.1</v>
-      </c>
-      <c r="O10" s="10">
         <v>15.8</v>
       </c>
-      <c r="P10" s="13">
+      <c r="N10" s="13">
         <v>69</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>2018</v>
       </c>
-      <c r="B11" s="7">
-        <v>1</v>
+      <c r="B11" s="6">
+        <v>0.2</v>
       </c>
       <c r="C11" s="6">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="D11" s="6">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="E11" s="6">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="F11" s="6">
-        <v>0.5</v>
+        <v>1.3</v>
       </c>
       <c r="G11" s="6">
-        <v>0.8</v>
+        <v>2.1</v>
       </c>
       <c r="H11" s="6">
-        <v>1.3</v>
+        <v>2.8</v>
       </c>
       <c r="I11" s="6">
-        <v>2.1</v>
+        <v>3.5</v>
       </c>
       <c r="J11" s="6">
-        <v>2.8</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="K11" s="6">
-        <v>3.5</v>
-      </c>
-      <c r="L11" s="6">
-        <v>4.5999999999999996</v>
+        <v>6.8</v>
+      </c>
+      <c r="L11" s="7">
+        <v>10</v>
       </c>
       <c r="M11" s="6">
-        <v>6.8</v>
-      </c>
-      <c r="N11" s="7">
-        <v>10</v>
-      </c>
-      <c r="O11" s="6">
         <v>15.9</v>
       </c>
-      <c r="P11" s="8">
+      <c r="N11" s="8">
         <v>67.7</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>2019</v>
       </c>
-      <c r="B12" s="7">
-        <v>1</v>
+      <c r="B12" s="6">
+        <v>0.2</v>
       </c>
       <c r="C12" s="6">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D12" s="6">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="E12" s="6">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="F12" s="6">
-        <v>0.5</v>
-      </c>
-      <c r="G12" s="6">
-        <v>0.7</v>
+        <v>1.2</v>
+      </c>
+      <c r="G12" s="7">
+        <v>2</v>
       </c>
       <c r="H12" s="6">
-        <v>1.2</v>
-      </c>
-      <c r="I12" s="7">
-        <v>2</v>
+        <v>2.7</v>
+      </c>
+      <c r="I12" s="6">
+        <v>3.4</v>
       </c>
       <c r="J12" s="6">
-        <v>2.7</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="K12" s="6">
-        <v>3.4</v>
+        <v>6.7</v>
       </c>
       <c r="L12" s="6">
-        <v>4.5999999999999996</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="M12" s="6">
-        <v>6.7</v>
-      </c>
-      <c r="N12" s="6">
-        <v>9.8000000000000007</v>
-      </c>
-      <c r="O12" s="6">
         <v>15.2</v>
       </c>
-      <c r="P12" s="9">
+      <c r="N12" s="9">
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>2020</v>
       </c>
       <c r="B13" s="6">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="C13" s="6">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D13" s="6">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="E13" s="6">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="F13" s="6">
-        <v>0.5</v>
+        <v>1.3</v>
       </c>
       <c r="G13" s="6">
-        <v>0.7</v>
+        <v>2.1</v>
       </c>
       <c r="H13" s="6">
-        <v>1.3</v>
+        <v>3.1</v>
       </c>
       <c r="I13" s="6">
-        <v>2.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="J13" s="6">
-        <v>3.1</v>
-      </c>
-      <c r="K13" s="6">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="L13" s="6">
         <v>5.5</v>
       </c>
-      <c r="M13" s="7">
+      <c r="K13" s="7">
         <v>8</v>
       </c>
-      <c r="N13" s="7">
+      <c r="L13" s="7">
         <v>12</v>
       </c>
-      <c r="O13" s="6">
+      <c r="M13" s="6">
         <v>18.8</v>
       </c>
-      <c r="P13" s="8">
+      <c r="N13" s="8">
         <v>75.5</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>2021</v>
       </c>
       <c r="B14" s="6">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="C14" s="6">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D14" s="6">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="E14" s="6">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="F14" s="6">
-        <v>0.5</v>
+        <v>1.4</v>
       </c>
       <c r="G14" s="6">
-        <v>0.8</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="H14" s="6">
-        <v>1.4</v>
+        <v>3.3</v>
       </c>
       <c r="I14" s="6">
-        <v>2.2000000000000002</v>
+        <v>4.5</v>
       </c>
       <c r="J14" s="6">
-        <v>3.3</v>
+        <v>6.2</v>
       </c>
       <c r="K14" s="6">
-        <v>4.5</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="L14" s="6">
-        <v>6.2</v>
+        <v>15.1</v>
       </c>
       <c r="M14" s="6">
-        <v>9.8000000000000007</v>
-      </c>
-      <c r="N14" s="6">
-        <v>15.1</v>
-      </c>
-      <c r="O14" s="6">
         <v>23.9</v>
       </c>
-      <c r="P14" s="9">
+      <c r="N14" s="9">
         <v>90</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>2022</v>
       </c>
       <c r="B15" s="6">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="C15" s="6">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D15" s="6">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="E15" s="6">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="F15" s="6">
-        <v>0.5</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="G15" s="6">
-        <v>0.6</v>
+        <v>1.8</v>
       </c>
       <c r="H15" s="6">
-        <v>1.1000000000000001</v>
+        <v>2.8</v>
       </c>
       <c r="I15" s="6">
-        <v>1.8</v>
+        <v>3.7</v>
       </c>
       <c r="J15" s="6">
-        <v>2.8</v>
+        <v>4.8</v>
       </c>
       <c r="K15" s="6">
-        <v>3.7</v>
+        <v>6.8</v>
       </c>
       <c r="L15" s="6">
-        <v>4.8</v>
+        <v>10.1</v>
       </c>
       <c r="M15" s="6">
-        <v>6.8</v>
-      </c>
-      <c r="N15" s="6">
-        <v>10.1</v>
-      </c>
-      <c r="O15" s="6">
         <v>15.6</v>
       </c>
-      <c r="P15" s="8">
+      <c r="N15" s="8">
         <v>66.3</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>2023</v>
       </c>
       <c r="B16" s="6">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="C16" s="6">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D16" s="6">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E16" s="6">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="F16" s="6">
-        <v>0.4</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="G16" s="6">
-        <v>0.6</v>
+        <v>1.7</v>
       </c>
       <c r="H16" s="6">
-        <v>1.1000000000000001</v>
+        <v>2.7</v>
       </c>
       <c r="I16" s="6">
-        <v>1.7</v>
+        <v>3.6</v>
       </c>
       <c r="J16" s="6">
-        <v>2.7</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="K16" s="6">
-        <v>3.6</v>
+        <v>6.4</v>
       </c>
       <c r="L16" s="6">
-        <v>4.5999999999999996</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="M16" s="6">
-        <v>6.4</v>
-      </c>
-      <c r="N16" s="6">
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="O16" s="6">
         <v>13.9</v>
       </c>
-      <c r="P16" s="8">
+      <c r="N16" s="8">
         <v>57.5</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -6533,12 +6341,10 @@
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>